<commit_message>
Keep per-exercise drafts, add 0-10 effort scale, migrate old data
- Edited values in an exercise form persist for the day (across switching
  exercises and reloads), with an "изменено" badge and a reset-to-default button
- Replace easy/ok/hard with a 0-10 effort slider; 8+ repeats load, 4 and below
  adds reps; shown in the diary and exported to Excel
- Migrate stored entries and drafts from the old feel field to effort on load
- Jump-to-week reset and full reset in the plan view

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example-export.xlsx
+++ b/example-export.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="60">
   <si>
     <t>ДНЕВНИК ТРЕНИРОВОК</t>
   </si>
   <si>
-    <t>ВЫГРУЖЕНО 12.10.2026 · ЗАПИСЕЙ: 2 · БОЛЬ 4 И ВЫШЕ — СНИЖАЕМ НАГРУЗКУ</t>
+    <t>ВЫГРУЖЕНО 16.10.2026 · ЗАПИСЕЙ: 2 · БОЛЬ 4 И ВЫШЕ — СНИЖАЕМ НАГРУЗКУ</t>
   </si>
   <si>
     <t>ДАТА</t>
@@ -42,7 +42,7 @@
     <t>БОЛЬ В СПИНЕ</t>
   </si>
   <si>
-    <t>КАК ПОШЛО</t>
+    <t>СЛОЖНОСТЬ (0–10)</t>
   </si>
   <si>
     <t>ОБЪЁМ, КГ</t>
@@ -54,18 +54,12 @@
     <t>Жим штанги лёжа</t>
   </si>
   <si>
-    <t>Тяжело</t>
-  </si>
-  <si>
     <t>Легко, технику держал</t>
   </si>
   <si>
     <t>Планка (сек)</t>
   </si>
   <si>
-    <t>Норм</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -78,7 +72,7 @@
     <t>РАБОЧИЕ ВЕСА</t>
   </si>
   <si>
-    <t>ОКРУГЛЕНИЕ ДО 2,5 КГ · 12.10.2026</t>
+    <t>ОКРУГЛЕНИЕ ДО 2,5 КГ · 16.10.2026</t>
   </si>
   <si>
     <t>ПОСЛЕДНИЙ ВЕС</t>
@@ -186,7 +180,7 @@
     <t>СВОДКА</t>
   </si>
   <si>
-    <t>ПО УПРАЖНЕНИЯМ · 12.10.2026</t>
+    <t>ПО УПРАЖНЕНИЯМ · 16.10.2026</t>
   </si>
   <si>
     <t>ТРЕНИРОВОК</t>
@@ -742,7 +736,7 @@
     <col min="4" max="4" width="10" style="3" customWidth="1"/>
     <col min="5" max="6" width="10" style="2" customWidth="1"/>
     <col min="7" max="7" width="13" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="16" style="2" customWidth="1"/>
     <col min="9" max="9" width="12" style="4" customWidth="1"/>
     <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
@@ -783,7 +777,7 @@
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="9"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="11"/>
       <c r="J3" s="9"/>
     </row>
@@ -809,7 +803,7 @@
       <c r="G4" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="13" t="s">
         <v>9</v>
       </c>
       <c r="I4" s="16" t="s">
@@ -841,15 +835,15 @@
       <c r="G5" s="21">
         <v>5</v>
       </c>
-      <c r="H5" s="19" t="s">
-        <v>13</v>
+      <c r="H5" s="18">
+        <v>9</v>
       </c>
       <c r="I5" s="22">
         <f>D5*E5*F5</f>
         <v>1080</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -860,7 +854,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" s="26">
         <v>0</v>
@@ -874,49 +868,49 @@
       <c r="G6" s="24">
         <v>0</v>
       </c>
-      <c r="H6" s="25" t="s">
-        <v>16</v>
+      <c r="H6" s="24">
+        <v>5</v>
       </c>
       <c r="I6" s="27">
         <f>D6*E6*F6</f>
         <v>0</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B7" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="30" t="s">
-        <v>19</v>
-      </c>
       <c r="D7" s="31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="29">
         <f>SUM(E5:E6)</f>
         <v>6</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G7" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>15</v>
       </c>
       <c r="I7" s="32">
         <f>SUM(I5:I6)</f>
         <v>1080</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -945,7 +939,7 @@
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="33" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -955,7 +949,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="34"/>
@@ -976,19 +970,19 @@
         <v>4</v>
       </c>
       <c r="B4" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="E4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="F4" s="14" t="s">
         <v>24</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -999,156 +993,156 @@
         <v>55</v>
       </c>
       <c r="C5" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="F5" s="19" t="s">
         <v>28</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B6" s="26">
         <v>55</v>
       </c>
       <c r="C6" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="F6" s="25" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="20">
         <v>115</v>
       </c>
       <c r="C7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="F7" s="19" t="s">
         <v>34</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" s="26">
         <v>45</v>
       </c>
       <c r="C8" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="25" t="s">
         <v>38</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="25" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B9" s="20">
         <v>45</v>
       </c>
       <c r="C9" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="19" t="s">
         <v>38</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B10" s="26">
         <v>20</v>
       </c>
       <c r="C10" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="F10" s="25" t="s">
         <v>44</v>
-      </c>
-      <c r="E10" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" s="25" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="19" t="s">
+      <c r="E11" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="F11" s="19" t="s">
         <v>49</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="25" t="s">
+      <c r="F12" s="25" t="s">
         <v>53</v>
-      </c>
-      <c r="E12" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="25" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1179,7 +1173,7 @@
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
@@ -1188,7 +1182,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B2" s="34"/>
       <c r="C2" s="34"/>
@@ -1207,13 +1201,13 @@
         <v>4</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>58</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>60</v>
       </c>
       <c r="E4" s="16" t="s">
         <v>10</v>
@@ -1238,7 +1232,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" s="24">
         <v>1</v>
@@ -1255,16 +1249,16 @@
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="32">
         <v>1080</v>

</xml_diff>